<commit_message>
fix(ods): a cell's runs take its style's and their paragraph style's looks
A spreadsheet sets a cell bold (or its font, size, colour) through the cell's style: its runs were
read from their own spans alone, so a bold header cell read plain, and its paragraph style was not
read either.
</commit_message>
<xml_diff>
--- a/test/generator/baseline/gen.ods.to.xlsx.xlsx
+++ b/test/generator/baseline/gen.ods.to.xlsx.xlsx
@@ -51,8 +51,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1" vertical="top"/>
     </xf>
@@ -193,14 +194,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Text Formatting </t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Inline formatting </t>
         </is>
@@ -242,7 +243,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Fun with fonts </t>
         </is>
@@ -256,7 +257,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Paragraph level formatting </t>
         </is>
@@ -270,7 +271,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">For the lovers of poetry amongst you, paragraphs with hanging indents, like this often
 come in handy. You can use hanging indents to ensure that a line of poetry retains its individual identity as a line even when the screen is  too narrow to display it as a single line. Not only does this paragraph have a hanging indent, it is also has an extra top margin, setting it apart from the preceding paragraph. </t>
@@ -293,19 +294,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Tables </t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">ITEM </t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">NEEDED </t>
         </is>
@@ -522,22 +523,22 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">College </t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">New students </t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Graduating students </t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Change </t>
         </is>
@@ -895,7 +896,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Structural Elements </t>
         </is>
@@ -909,7 +910,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Footnotes &amp; Endnotes </t>
         </is>
@@ -923,7 +924,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Dropcaps </t>
         </is>
@@ -944,7 +945,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Links </t>
         </is>
@@ -968,7 +969,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Images </t>
         </is>
@@ -1001,7 +1002,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Lists </t>
         </is>
@@ -1015,7 +1016,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Bulleted List </t>
         </is>
@@ -1036,7 +1037,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Numbered List </t>
         </is>
@@ -1063,7 +1064,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Multi-level Lists </t>
         </is>
@@ -1172,7 +1173,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Continued Lists </t>
         </is>
@@ -1249,7 +1250,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Charts</t>
         </is>

</xml_diff>